<commit_message>
US Courts F-2: fetch the confirmed three-month and twelve-month files and parse the AO layout
File names confirmed on the AO's per-table pages
(document/bf_f2.3_MMDD.YYYY.xlsx and bf_f2_MMDD.YYYY.xlsx). The parser
accepts the merged header rows (All Chapters, Chapter 7, 11, 13 under
Business and Nonbusiness), normalizes district labels such as OK,N and
maps the combined Arkansas row to fips 05. Sources may declare
fetch_all so the CLI ingests every candidate that parses.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HLvGmhQhGHbeRJyW3hB9qm
</commit_message>
<xml_diff>
--- a/ingest/tests/fixtures/uscourts_f2_synthetic.xlsx
+++ b/ingest/tests/fixtures/uscourts_f2_synthetic.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J12"/>
+  <dimension ref="A1:O14"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -426,336 +426,542 @@
     <row r="3">
       <c r="A3" t="inlineStr">
         <is>
+          <t>Predominant Nature of Debt</t>
+        </is>
+      </c>
+    </row>
+    <row r="4">
+      <c r="A4" t="inlineStr">
+        <is>
           <t>Circuit and District</t>
         </is>
       </c>
-      <c r="B3" t="inlineStr">
-        <is>
-          <t>Total Filings</t>
-        </is>
-      </c>
-      <c r="C3" t="inlineStr">
+      <c r="B4" t="inlineStr">
+        <is>
+          <t>Total</t>
+        </is>
+      </c>
+      <c r="G4" t="inlineStr">
         <is>
           <t>Business</t>
         </is>
       </c>
-      <c r="G3" t="inlineStr">
+      <c r="L4" t="inlineStr">
         <is>
           <t>Nonbusiness</t>
         </is>
       </c>
     </row>
-    <row r="4">
-      <c r="C4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="D4" t="inlineStr">
+    <row r="5">
+      <c r="B5" t="inlineStr">
+        <is>
+          <t>All Chapters</t>
+        </is>
+      </c>
+      <c r="C5" t="inlineStr">
         <is>
           <t>Chapter 7</t>
         </is>
       </c>
-      <c r="E4" t="inlineStr">
+      <c r="D5" t="inlineStr">
         <is>
           <t>Chapter 11</t>
         </is>
       </c>
-      <c r="F4" t="inlineStr">
+      <c r="E5" t="inlineStr">
         <is>
           <t>Chapter 13</t>
         </is>
       </c>
-      <c r="G4" t="inlineStr">
-        <is>
-          <t>Total</t>
-        </is>
-      </c>
-      <c r="H4" t="inlineStr">
+      <c r="F5" t="inlineStr">
+        <is>
+          <t>Other Chapters</t>
+        </is>
+      </c>
+      <c r="G5" t="inlineStr">
+        <is>
+          <t>All Chapters</t>
+        </is>
+      </c>
+      <c r="H5" t="inlineStr">
         <is>
           <t>Chapter 7</t>
         </is>
       </c>
-      <c r="I4" t="inlineStr">
+      <c r="I5" t="inlineStr">
         <is>
           <t>Chapter 11</t>
         </is>
       </c>
-      <c r="J4" t="inlineStr">
+      <c r="J5" t="inlineStr">
         <is>
           <t>Chapter 13</t>
         </is>
       </c>
-    </row>
-    <row r="5">
-      <c r="A5" t="inlineStr">
-        <is>
-          <t>TOTAL</t>
-        </is>
-      </c>
-      <c r="B5" t="n">
-        <v>9999</v>
-      </c>
-      <c r="C5" t="n">
-        <v>100</v>
-      </c>
-      <c r="D5" t="n">
-        <v>50</v>
-      </c>
-      <c r="E5" t="n">
-        <v>20</v>
-      </c>
-      <c r="F5" t="n">
-        <v>30</v>
-      </c>
-      <c r="G5" t="n">
-        <v>9899</v>
-      </c>
-      <c r="H5" t="n">
-        <v>6000</v>
-      </c>
-      <c r="I5" t="n">
-        <v>9</v>
-      </c>
-      <c r="J5" t="n">
-        <v>3890</v>
+      <c r="K5" t="inlineStr">
+        <is>
+          <t>Other Chapters</t>
+        </is>
+      </c>
+      <c r="L5" t="inlineStr">
+        <is>
+          <t>All Chapters</t>
+        </is>
+      </c>
+      <c r="M5" t="inlineStr">
+        <is>
+          <t>Chapter 7</t>
+        </is>
+      </c>
+      <c r="N5" t="inlineStr">
+        <is>
+          <t>Chapter 11</t>
+        </is>
+      </c>
+      <c r="O5" t="inlineStr">
+        <is>
+          <t>Chapter 13</t>
+        </is>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="inlineStr">
         <is>
-          <t>10TH</t>
+          <t>Total</t>
         </is>
       </c>
       <c r="B6" t="n">
-        <v>500</v>
+        <v>9999</v>
       </c>
       <c r="C6" t="n">
-        <v>10</v>
+        <v>6100</v>
       </c>
       <c r="D6" t="n">
-        <v>5</v>
+        <v>29</v>
       </c>
       <c r="E6" t="n">
-        <v>2</v>
+        <v>3920</v>
       </c>
       <c r="F6" t="n">
-        <v>3</v>
+        <v>0</v>
       </c>
       <c r="G6" t="n">
-        <v>490</v>
+        <v>100</v>
       </c>
       <c r="H6" t="n">
-        <v>300</v>
+        <v>50</v>
       </c>
       <c r="I6" t="n">
-        <v>1</v>
+        <v>20</v>
       </c>
       <c r="J6" t="n">
-        <v>189</v>
+        <v>30</v>
+      </c>
+      <c r="K6" t="n">
+        <v>0</v>
+      </c>
+      <c r="L6" t="n">
+        <v>9899</v>
+      </c>
+      <c r="M6" t="n">
+        <v>6000</v>
+      </c>
+      <c r="N6" t="n">
+        <v>9</v>
+      </c>
+      <c r="O6" t="n">
+        <v>3890</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="inlineStr">
         <is>
-          <t>OKN</t>
+          <t>10th</t>
         </is>
       </c>
       <c r="B7" t="n">
-        <v>120</v>
+        <v>500</v>
       </c>
       <c r="C7" t="n">
+        <v>310</v>
+      </c>
+      <c r="D7" t="n">
+        <v>3</v>
+      </c>
+      <c r="E7" t="n">
+        <v>192</v>
+      </c>
+      <c r="F7" t="n">
+        <v>0</v>
+      </c>
+      <c r="G7" t="n">
+        <v>10</v>
+      </c>
+      <c r="H7" t="n">
+        <v>5</v>
+      </c>
+      <c r="I7" t="n">
         <v>2</v>
       </c>
-      <c r="D7" t="n">
-        <v>1</v>
-      </c>
-      <c r="E7" t="n">
-        <v>0</v>
-      </c>
-      <c r="F7" t="n">
-        <v>1</v>
-      </c>
-      <c r="G7" t="n">
-        <v>118</v>
-      </c>
-      <c r="H7" t="n">
-        <v>70</v>
-      </c>
-      <c r="I7" t="n">
-        <v>0</v>
-      </c>
       <c r="J7" t="n">
-        <v>48</v>
+        <v>3</v>
+      </c>
+      <c r="K7" t="n">
+        <v>0</v>
+      </c>
+      <c r="L7" t="n">
+        <v>490</v>
+      </c>
+      <c r="M7" t="n">
+        <v>300</v>
+      </c>
+      <c r="N7" t="n">
+        <v>1</v>
+      </c>
+      <c r="O7" t="n">
+        <v>189</v>
       </c>
     </row>
     <row r="8">
       <c r="A8" t="inlineStr">
         <is>
-          <t>OKE</t>
+          <t>OK,N</t>
         </is>
       </c>
       <c r="B8" t="n">
-        <v>80</v>
+        <v>120</v>
       </c>
       <c r="C8" t="n">
-        <v>1</v>
+        <v>71</v>
       </c>
       <c r="D8" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E8" t="n">
-        <v>0</v>
+        <v>49</v>
       </c>
       <c r="F8" t="n">
         <v>0</v>
       </c>
       <c r="G8" t="n">
-        <v>79</v>
+        <v>2</v>
       </c>
       <c r="H8" t="n">
-        <v>50</v>
+        <v>1</v>
       </c>
       <c r="I8" t="n">
         <v>0</v>
       </c>
       <c r="J8" t="n">
-        <v>29</v>
+        <v>1</v>
+      </c>
+      <c r="K8" t="n">
+        <v>0</v>
+      </c>
+      <c r="L8" t="n">
+        <v>118</v>
+      </c>
+      <c r="M8" t="n">
+        <v>70</v>
+      </c>
+      <c r="N8" t="n">
+        <v>0</v>
+      </c>
+      <c r="O8" t="n">
+        <v>48</v>
       </c>
     </row>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
-          <t>OKW</t>
+          <t>OK,E</t>
         </is>
       </c>
       <c r="B9" t="n">
-        <v>200</v>
+        <v>80</v>
       </c>
       <c r="C9" t="n">
-        <v>4</v>
+        <v>51</v>
       </c>
       <c r="D9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="E9" t="n">
-        <v>1</v>
+        <v>29</v>
       </c>
       <c r="F9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G9" t="n">
-        <v>196</v>
+        <v>1</v>
       </c>
       <c r="H9" t="n">
-        <v>120</v>
+        <v>1</v>
       </c>
       <c r="I9" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="J9" t="n">
-        <v>75</v>
+        <v>0</v>
+      </c>
+      <c r="K9" t="n">
+        <v>0</v>
+      </c>
+      <c r="L9" t="n">
+        <v>79</v>
+      </c>
+      <c r="M9" t="n">
+        <v>50</v>
+      </c>
+      <c r="N9" t="n">
+        <v>0</v>
+      </c>
+      <c r="O9" t="n">
+        <v>29</v>
       </c>
     </row>
     <row r="10">
       <c r="A10" t="inlineStr">
         <is>
-          <t>KS</t>
+          <t>OK,W</t>
         </is>
       </c>
       <c r="B10" t="n">
-        <v>150</v>
+        <v>200</v>
       </c>
       <c r="C10" t="n">
-        <v>3</v>
+        <v>122</v>
       </c>
       <c r="D10" t="n">
-        <v>1</v>
+        <v>2</v>
       </c>
       <c r="E10" t="n">
-        <v>1</v>
+        <v>76</v>
       </c>
       <c r="F10" t="n">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="G10" t="n">
-        <v>147</v>
+        <v>4</v>
       </c>
       <c r="H10" t="n">
-        <v>90</v>
+        <v>2</v>
       </c>
       <c r="I10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J10" t="n">
-        <v>57</v>
+        <v>1</v>
+      </c>
+      <c r="K10" t="n">
+        <v>0</v>
+      </c>
+      <c r="L10" t="n">
+        <v>196</v>
+      </c>
+      <c r="M10" t="n">
+        <v>120</v>
+      </c>
+      <c r="N10" t="n">
+        <v>1</v>
+      </c>
+      <c r="O10" t="n">
+        <v>75</v>
       </c>
     </row>
     <row r="11">
       <c r="A11" t="inlineStr">
         <is>
-          <t>3RD</t>
+          <t>KS</t>
         </is>
       </c>
       <c r="B11" t="n">
-        <v>300</v>
+        <v>150</v>
       </c>
       <c r="C11" t="n">
-        <v>5</v>
+        <v>91</v>
       </c>
       <c r="D11" t="n">
-        <v>2</v>
+        <v>1</v>
       </c>
       <c r="E11" t="n">
-        <v>1</v>
+        <v>58</v>
       </c>
       <c r="F11" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="G11" t="n">
-        <v>295</v>
+        <v>3</v>
       </c>
       <c r="H11" t="n">
-        <v>200</v>
+        <v>1</v>
       </c>
       <c r="I11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="J11" t="n">
-        <v>95</v>
+        <v>1</v>
+      </c>
+      <c r="K11" t="n">
+        <v>0</v>
+      </c>
+      <c r="L11" t="n">
+        <v>147</v>
+      </c>
+      <c r="M11" t="n">
+        <v>90</v>
+      </c>
+      <c r="N11" t="n">
+        <v>0</v>
+      </c>
+      <c r="O11" t="n">
+        <v>57</v>
       </c>
     </row>
     <row r="12">
       <c r="A12" t="inlineStr">
         <is>
+          <t>AR</t>
+        </is>
+      </c>
+      <c r="B12" t="n">
+        <v>100</v>
+      </c>
+      <c r="C12" t="n">
+        <v>60</v>
+      </c>
+      <c r="D12" t="n">
+        <v>1</v>
+      </c>
+      <c r="E12" t="n">
+        <v>39</v>
+      </c>
+      <c r="F12" t="n">
+        <v>0</v>
+      </c>
+      <c r="G12" t="n">
+        <v>2</v>
+      </c>
+      <c r="H12" t="n">
+        <v>1</v>
+      </c>
+      <c r="I12" t="n">
+        <v>0</v>
+      </c>
+      <c r="J12" t="n">
+        <v>1</v>
+      </c>
+      <c r="K12" t="n">
+        <v>0</v>
+      </c>
+      <c r="L12" t="n">
+        <v>98</v>
+      </c>
+      <c r="M12" t="n">
+        <v>59</v>
+      </c>
+      <c r="N12" t="n">
+        <v>1</v>
+      </c>
+      <c r="O12" t="n">
+        <v>38</v>
+      </c>
+    </row>
+    <row r="13">
+      <c r="A13" t="inlineStr">
+        <is>
+          <t>3rd</t>
+        </is>
+      </c>
+      <c r="B13" t="n">
+        <v>300</v>
+      </c>
+      <c r="C13" t="n">
+        <v>202</v>
+      </c>
+      <c r="D13" t="n">
+        <v>1</v>
+      </c>
+      <c r="E13" t="n">
+        <v>97</v>
+      </c>
+      <c r="F13" t="n">
+        <v>0</v>
+      </c>
+      <c r="G13" t="n">
+        <v>5</v>
+      </c>
+      <c r="H13" t="n">
+        <v>2</v>
+      </c>
+      <c r="I13" t="n">
+        <v>1</v>
+      </c>
+      <c r="J13" t="n">
+        <v>2</v>
+      </c>
+      <c r="K13" t="n">
+        <v>0</v>
+      </c>
+      <c r="L13" t="n">
+        <v>295</v>
+      </c>
+      <c r="M13" t="n">
+        <v>200</v>
+      </c>
+      <c r="N13" t="n">
+        <v>0</v>
+      </c>
+      <c r="O13" t="n">
+        <v>95</v>
+      </c>
+    </row>
+    <row r="14">
+      <c r="A14" t="inlineStr">
+        <is>
           <t>NJ</t>
         </is>
       </c>
-      <c r="B12" t="n">
+      <c r="B14" t="n">
         <v>300</v>
       </c>
-      <c r="C12" t="n">
+      <c r="C14" t="n">
+        <v>202</v>
+      </c>
+      <c r="D14" t="n">
+        <v>1</v>
+      </c>
+      <c r="E14" t="n">
+        <v>97</v>
+      </c>
+      <c r="F14" t="n">
+        <v>0</v>
+      </c>
+      <c r="G14" t="n">
         <v>5</v>
       </c>
-      <c r="D12" t="n">
+      <c r="H14" t="n">
         <v>2</v>
       </c>
-      <c r="E12" t="n">
-        <v>1</v>
-      </c>
-      <c r="F12" t="n">
+      <c r="I14" t="n">
+        <v>1</v>
+      </c>
+      <c r="J14" t="n">
         <v>2</v>
       </c>
-      <c r="G12" t="n">
+      <c r="K14" t="n">
+        <v>0</v>
+      </c>
+      <c r="L14" t="n">
         <v>295</v>
       </c>
-      <c r="H12" t="n">
+      <c r="M14" t="n">
         <v>200</v>
       </c>
-      <c r="I12" t="n">
-        <v>0</v>
-      </c>
-      <c r="J12" t="n">
+      <c r="N14" t="n">
+        <v>0</v>
+      </c>
+      <c r="O14" t="n">
         <v>95</v>
       </c>
     </row>

</xml_diff>

<commit_message>
F-2 parser: only two-letter district labels are rows; fixes North Dakota carrying the Second Circuit total
Stripping non-letters turned the circuit label 2nd into ND. District
labels are now matched as two letters with an optional division letter.
Rows regenerated from the archived June 2026 spreadsheets with the
runner's provenance carried over; North Dakota is 254 nonbusiness
filings for the quarter and 808 for the twelve months, as in the sheet.

Co-Authored-By: Claude Fable 5.1 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01HLvGmhQhGHbeRJyW3hB9qm
</commit_message>
<xml_diff>
--- a/ingest/tests/fixtures/uscourts_f2_synthetic.xlsx
+++ b/ingest/tests/fixtures/uscourts_f2_synthetic.xlsx
@@ -413,7 +413,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:O14"/>
+  <dimension ref="A1:O16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -965,6 +965,104 @@
         <v>95</v>
       </c>
     </row>
+    <row r="15">
+      <c r="A15" t="inlineStr">
+        <is>
+          <t xml:space="preserve">     2nd</t>
+        </is>
+      </c>
+      <c r="B15" t="n">
+        <v>7000</v>
+      </c>
+      <c r="C15" t="n">
+        <v>5000</v>
+      </c>
+      <c r="D15" t="n">
+        <v>200</v>
+      </c>
+      <c r="E15" t="n">
+        <v>1800</v>
+      </c>
+      <c r="F15" t="n">
+        <v>0</v>
+      </c>
+      <c r="G15" t="n">
+        <v>600</v>
+      </c>
+      <c r="H15" t="n">
+        <v>300</v>
+      </c>
+      <c r="I15" t="n">
+        <v>250</v>
+      </c>
+      <c r="J15" t="n">
+        <v>50</v>
+      </c>
+      <c r="K15" t="n">
+        <v>0</v>
+      </c>
+      <c r="L15" t="n">
+        <v>6400</v>
+      </c>
+      <c r="M15" t="n">
+        <v>4700</v>
+      </c>
+      <c r="N15" t="n">
+        <v>20</v>
+      </c>
+      <c r="O15" t="n">
+        <v>1680</v>
+      </c>
+    </row>
+    <row r="16">
+      <c r="A16" t="inlineStr">
+        <is>
+          <t>ND</t>
+        </is>
+      </c>
+      <c r="B16" t="n">
+        <v>268</v>
+      </c>
+      <c r="C16" t="n">
+        <v>228</v>
+      </c>
+      <c r="D16" t="n">
+        <v>3</v>
+      </c>
+      <c r="E16" t="n">
+        <v>36</v>
+      </c>
+      <c r="F16" t="n">
+        <v>1</v>
+      </c>
+      <c r="G16" t="n">
+        <v>14</v>
+      </c>
+      <c r="H16" t="n">
+        <v>10</v>
+      </c>
+      <c r="I16" t="n">
+        <v>3</v>
+      </c>
+      <c r="J16" t="n">
+        <v>0</v>
+      </c>
+      <c r="K16" t="n">
+        <v>1</v>
+      </c>
+      <c r="L16" t="n">
+        <v>254</v>
+      </c>
+      <c r="M16" t="n">
+        <v>218</v>
+      </c>
+      <c r="N16" t="n">
+        <v>0</v>
+      </c>
+      <c r="O16" t="n">
+        <v>36</v>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>